<commit_message>
Add capacity check and set 800 employees / Group II default in Betreuung calculator
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCKnGiGtYBiYx7scvoQXDr
</commit_message>
<xml_diff>
--- a/safety/betreuung_calculator_2027.xlsx
+++ b/safety/betreuung_calculator_2027.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="71">
   <si>
     <t xml:space="preserve">FaSi &amp; Betriebsarzt Betreuung – Grund- und Betriebsspezifische Betreuung</t>
   </si>
@@ -74,7 +74,7 @@
     <t xml:space="preserve">of which Betriebsarzt (h)</t>
   </si>
   <si>
-    <t xml:space="preserve">Warehouse / logistics</t>
+    <t xml:space="preserve">Warehouse (WZ 52.10)</t>
   </si>
   <si>
     <t xml:space="preserve">52.10</t>
@@ -83,91 +83,133 @@
     <t xml:space="preserve">II</t>
   </si>
   <si>
-    <t xml:space="preserve">Office / admin</t>
+    <t xml:space="preserve">Total Grundbetreuung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Betriebsspezifische Betreuung (hours per driver, from site needs assessment)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Driver / topic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FaSi (h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Betriebsarzt (h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basis / comment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gefährdungsbeurteilung updates &amp; audits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example – overwrite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arbeitsmedizinische Vorsorge (G25, G37, etc.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASA meetings &amp; site walkthroughs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projects: new equipment / layout changes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ergonomics, manual handling programme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Betriebsspezifische Betreuung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total (h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grundbetreuung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Betriebsspezifische Betreuung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gesamtbetreuung (h per year)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FTE equivalent (at productive h per FTE, see Reference)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gesamtbetreuung per employee (h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Betriebsspezifisch as % of Gesamtbetreuung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Capacity check (qualified staff vs required hours)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qualified FaSi (with Fachkunde) available to this site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source: user (3 FaSi on 40 h contracts). Unqualified staff are excluded.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contract hours per week per FaSi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source: user.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share of FaSi time allocated to this site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumption: 100 % – reduce if FaSi cover other sites.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Betriebsarzt hours quoted / contracted (TBC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter when the Betriebsarzt/provider quote is received.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FaSi capacity (h per year) = qualified FaSi x contract h / 40 x productive h per FTE x site share</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FaSi hours required (Gesamtbetreuung)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FaSi capacity surplus / (shortfall)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required FaSi hours as % of capacity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Betriebsarzt hours required (Gesamtbetreuung)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Betriebsarzt quote surplus / (shortfall)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference – DGUV Vorschrift 2, Anlage 2 (Betreuungsgruppen, Grundbetreuung)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Betreuungsgruppe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risk level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grundbetreuung (h per employee per year)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medium</t>
   </si>
   <si>
     <t xml:space="preserve">III</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Grundbetreuung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Betriebsspezifische Betreuung (hours per driver, from site needs assessment)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Driver / topic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FaSi (h)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Betriebsarzt (h)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Basis / comment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gefährdungsbeurteilung updates &amp; audits</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example – overwrite</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arbeitsmedizinische Vorsorge (G25, G37, etc.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ASA meetings &amp; site walkthroughs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Projects: new equipment / layout changes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ergonomics, manual handling programme</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Betriebsspezifische Betreuung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total (h)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grundbetreuung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Betriebsspezifische Betreuung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gesamtbetreuung (h per year)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FTE equivalent (at productive h per FTE, see Reference)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gesamtbetreuung per employee (h)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Betriebsspezifisch as % of Gesamtbetreuung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference – DGUV Vorschrift 2, Anlage 2 (Betreuungsgruppen, Grundbetreuung)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Betreuungsgruppe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Risk level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grundbetreuung (h per employee per year)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I</t>
-  </si>
-  <si>
-    <t xml:space="preserve">High</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medium</t>
   </si>
   <si>
     <t xml:space="preserve">Low</t>
@@ -354,7 +396,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -441,6 +483,14 @@
     </xf>
     <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
@@ -715,7 +765,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -879,7 +929,7 @@
         <v>19</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>250</v>
+        <v>800</v>
       </c>
       <c r="E11" s="12" t="n">
         <f aca="false">IF(C11="","",INDEX(Reference!$C$4:$C$6,MATCH(C11,Reference!$A$4:$A$6,0)))</f>
@@ -887,43 +937,37 @@
       </c>
       <c r="F11" s="13" t="n">
         <f aca="false">IF(C11="",0,D11*E11)</f>
-        <v>375</v>
+        <v>1200</v>
       </c>
       <c r="G11" s="13" t="n">
         <f aca="false">F11*$B$6</f>
-        <v>187.5</v>
+        <v>600</v>
       </c>
       <c r="H11" s="13" t="n">
         <f aca="false">F11*$B$7</f>
-        <v>187.5</v>
+        <v>600</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
-        <v>20</v>
-      </c>
+      <c r="A12" s="5"/>
       <c r="B12" s="5"/>
-      <c r="C12" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="D12" s="11" t="n">
-        <v>40</v>
-      </c>
-      <c r="E12" s="12" t="n">
+      <c r="C12" s="10"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="12" t="str">
         <f aca="false">IF(C12="","",INDEX(Reference!$C$4:$C$6,MATCH(C12,Reference!$A$4:$A$6,0)))</f>
-        <v>0.5</v>
+        <v/>
       </c>
       <c r="F12" s="13" t="n">
         <f aca="false">IF(C12="",0,D12*E12)</f>
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="G12" s="13" t="n">
         <f aca="false">F12*$B$6</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H12" s="13" t="n">
         <f aca="false">F12*$B$7</f>
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1104,29 +1148,29 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B21" s="14"/>
       <c r="C21" s="14"/>
       <c r="D21" s="15" t="n">
         <f aca="false">SUM(D11:D20)</f>
-        <v>290</v>
+        <v>800</v>
       </c>
       <c r="E21" s="16" t="n">
         <f aca="false">IF(D21=0,0,F21/D21)</f>
-        <v>1.36206896551724</v>
+        <v>1.5</v>
       </c>
       <c r="F21" s="17" t="n">
         <f aca="false">SUM(F11:F20)</f>
-        <v>395</v>
+        <v>1200</v>
       </c>
       <c r="G21" s="17" t="n">
         <f aca="false">SUM(G11:G20)</f>
-        <v>197.5</v>
+        <v>600</v>
       </c>
       <c r="H21" s="17" t="n">
         <f aca="false">SUM(H11:H20)</f>
-        <v>197.5</v>
+        <v>600</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1141,7 +1185,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -1153,25 +1197,25 @@
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B24" s="9"/>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
       <c r="F24" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="G24" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="H24" s="9" t="s">
         <v>25</v>
-      </c>
-      <c r="G24" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H24" s="9" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -1184,12 +1228,12 @@
         <v>0</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
@@ -1202,12 +1246,12 @@
         <v>80</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -1220,12 +1264,12 @@
         <v>12</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -1238,12 +1282,12 @@
         <v>8</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -1256,7 +1300,7 @@
         <v>20</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1291,7 +1335,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
@@ -1337,18 +1381,18 @@
       <c r="D36" s="9"/>
       <c r="E36" s="9"/>
       <c r="F36" s="9" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G36" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="19" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B37" s="19"/>
       <c r="C37" s="19"/>
@@ -1356,20 +1400,20 @@
       <c r="E37" s="19"/>
       <c r="F37" s="13" t="n">
         <f aca="false">G21</f>
-        <v>197.5</v>
+        <v>600</v>
       </c>
       <c r="G37" s="13" t="n">
         <f aca="false">H21</f>
-        <v>197.5</v>
+        <v>600</v>
       </c>
       <c r="H37" s="13" t="n">
         <f aca="false">F37+G37</f>
-        <v>395</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="19" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B38" s="19"/>
       <c r="C38" s="19"/>
@@ -1390,7 +1434,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="14" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B39" s="14"/>
       <c r="C39" s="14"/>
@@ -1398,20 +1442,20 @@
       <c r="E39" s="14"/>
       <c r="F39" s="17" t="n">
         <f aca="false">SUM(F37:F38)</f>
-        <v>341.5</v>
+        <v>744</v>
       </c>
       <c r="G39" s="17" t="n">
         <f aca="false">SUM(G37:G38)</f>
-        <v>317.5</v>
+        <v>720</v>
       </c>
       <c r="H39" s="17" t="n">
         <f aca="false">SUM(H37:H38)</f>
-        <v>659</v>
+        <v>1464</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="19" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B40" s="19"/>
       <c r="C40" s="19"/>
@@ -1419,20 +1463,20 @@
       <c r="E40" s="19"/>
       <c r="F40" s="20" t="n">
         <f aca="false">F39/Reference!$C$9</f>
-        <v>0.2134375</v>
+        <v>0.465</v>
       </c>
       <c r="G40" s="20" t="n">
         <f aca="false">G39/Reference!$C$9</f>
-        <v>0.1984375</v>
+        <v>0.45</v>
       </c>
       <c r="H40" s="20" t="n">
         <f aca="false">H39/Reference!$C$9</f>
-        <v>0.411875</v>
+        <v>0.915</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="19" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B41" s="19"/>
       <c r="C41" s="19"/>
@@ -1442,12 +1486,12 @@
       <c r="G41" s="19"/>
       <c r="H41" s="20" t="n">
         <f aca="false">IF(D21=0,0,H39/D21)</f>
-        <v>2.27241379310345</v>
+        <v>1.83</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="19" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B42" s="19"/>
       <c r="C42" s="19"/>
@@ -1455,15 +1499,15 @@
       <c r="E42" s="19"/>
       <c r="F42" s="21" t="n">
         <f aca="false">IF(F39=0,0,F38/F39)</f>
-        <v>0.421669106881406</v>
+        <v>0.193548387096774</v>
       </c>
       <c r="G42" s="21" t="n">
         <f aca="false">IF(G39=0,0,G38/G39)</f>
-        <v>0.377952755905512</v>
+        <v>0.166666666666667</v>
       </c>
       <c r="H42" s="21" t="n">
         <f aca="false">IF(H39=0,0,H38/H39)</f>
-        <v>0.400606980273141</v>
+        <v>0.180327868852459</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1476,8 +1520,218 @@
       <c r="G43" s="2"/>
       <c r="H43" s="2"/>
     </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B44" s="2"/>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="2"/>
+      <c r="H44" s="2"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B45" s="22"/>
+      <c r="C45" s="22"/>
+      <c r="D45" s="22"/>
+      <c r="E45" s="22"/>
+      <c r="F45" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G45" s="2"/>
+      <c r="H45" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="B46" s="22"/>
+      <c r="C46" s="22"/>
+      <c r="D46" s="22"/>
+      <c r="E46" s="22"/>
+      <c r="F46" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="G46" s="2"/>
+      <c r="H46" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="B47" s="22"/>
+      <c r="C47" s="22"/>
+      <c r="D47" s="22"/>
+      <c r="E47" s="22"/>
+      <c r="F47" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="2"/>
+      <c r="H47" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="22" t="s">
+        <v>47</v>
+      </c>
+      <c r="B48" s="22"/>
+      <c r="C48" s="22"/>
+      <c r="D48" s="22"/>
+      <c r="E48" s="22"/>
+      <c r="F48" s="18"/>
+      <c r="G48" s="2"/>
+      <c r="H48" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="B49" s="23"/>
+      <c r="C49" s="23"/>
+      <c r="D49" s="23"/>
+      <c r="E49" s="23"/>
+      <c r="F49" s="13" t="n">
+        <f aca="false">F45*F46/40*Reference!$C$9*F47</f>
+        <v>4800</v>
+      </c>
+      <c r="G49" s="19"/>
+      <c r="H49" s="19"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="B50" s="19"/>
+      <c r="C50" s="19"/>
+      <c r="D50" s="19"/>
+      <c r="E50" s="19"/>
+      <c r="F50" s="13" t="n">
+        <f aca="false">F39</f>
+        <v>744</v>
+      </c>
+      <c r="G50" s="19"/>
+      <c r="H50" s="19"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="B51" s="19"/>
+      <c r="C51" s="19"/>
+      <c r="D51" s="19"/>
+      <c r="E51" s="19"/>
+      <c r="F51" s="13" t="n">
+        <f aca="false">F49-F50</f>
+        <v>4056</v>
+      </c>
+      <c r="G51" s="19"/>
+      <c r="H51" s="19" t="str">
+        <f aca="false">IF(F51&gt;=0,"OK – required hours covered by qualified FaSi","SHORTFALL – needs additional FaSi time")</f>
+        <v>OK – required hours covered by qualified FaSi</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="B52" s="19"/>
+      <c r="C52" s="19"/>
+      <c r="D52" s="19"/>
+      <c r="E52" s="19"/>
+      <c r="F52" s="21" t="n">
+        <f aca="false">IF(F49=0,0,F50/F49)</f>
+        <v>0.155</v>
+      </c>
+      <c r="G52" s="19"/>
+      <c r="H52" s="19"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="B53" s="19"/>
+      <c r="C53" s="19"/>
+      <c r="D53" s="19"/>
+      <c r="E53" s="19"/>
+      <c r="F53" s="13" t="n">
+        <f aca="false">G39</f>
+        <v>720</v>
+      </c>
+      <c r="G53" s="19"/>
+      <c r="H53" s="19"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="B54" s="19"/>
+      <c r="C54" s="19"/>
+      <c r="D54" s="19"/>
+      <c r="E54" s="19"/>
+      <c r="F54" s="13" t="str">
+        <f aca="false">IF(F48="","",F48-F53)</f>
+        <v/>
+      </c>
+      <c r="G54" s="19"/>
+      <c r="H54" s="19" t="str">
+        <f aca="false">IF(F48="","Awaiting Betriebsarzt quote",IF(F54&gt;=0,"OK – quote covers required hours","SHORTFALL – quote below required hours"))</f>
+        <v>Awaiting Betriebsarzt quote</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="2"/>
+      <c r="B55" s="2"/>
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="2"/>
+      <c r="F55" s="2"/>
+      <c r="G55" s="2"/>
+      <c r="H55" s="2"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="2"/>
+      <c r="B56" s="2"/>
+      <c r="C56" s="2"/>
+      <c r="D56" s="2"/>
+      <c r="E56" s="2"/>
+      <c r="F56" s="2"/>
+      <c r="G56" s="2"/>
+      <c r="H56" s="2"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="2"/>
+      <c r="B57" s="2"/>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="2"/>
+      <c r="H57" s="2"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="2"/>
+      <c r="B58" s="2"/>
+      <c r="C58" s="2"/>
+      <c r="D58" s="2"/>
+      <c r="E58" s="2"/>
+      <c r="F58" s="2"/>
+      <c r="G58" s="2"/>
+      <c r="H58" s="2"/>
+    </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="25">
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A26:E26"/>
     <mergeCell ref="A27:E27"/>
@@ -1493,6 +1747,16 @@
     <mergeCell ref="A40:E40"/>
     <mergeCell ref="A41:E41"/>
     <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A45:E45"/>
+    <mergeCell ref="A46:E46"/>
+    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A48:E48"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="A51:E51"/>
+    <mergeCell ref="A52:E52"/>
+    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="A54:E54"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C11:C20" type="list">
@@ -1525,7 +1789,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1537,45 +1801,45 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="B4" s="22" t="s">
-        <v>47</v>
-      </c>
-      <c r="C4" s="23" t="n">
+      <c r="A4" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="25" t="n">
         <v>2.5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="22" t="s">
-        <v>48</v>
-      </c>
-      <c r="C5" s="23" t="n">
+      <c r="B5" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="25" t="n">
         <v>1.5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="22" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" s="22" t="s">
-        <v>49</v>
-      </c>
-      <c r="C6" s="23" t="n">
+      <c r="A6" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" s="25" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -1586,19 +1850,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="B8" s="2"/>
-      <c r="C8" s="24" t="n">
+      <c r="C8" s="26" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="B9" s="2"/>
-      <c r="C9" s="25" t="n">
+      <c r="C9" s="27" t="n">
         <v>1600</v>
       </c>
     </row>
@@ -1609,38 +1873,38 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="26" t="s">
-        <v>53</v>
-      </c>
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
+      <c r="A12" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" s="28"/>
+      <c r="C12" s="28"/>
     </row>
     <row r="13" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="26" t="s">
-        <v>54</v>
-      </c>
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
+      <c r="A13" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="B13" s="28"/>
+      <c r="C13" s="28"/>
     </row>
     <row r="14" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="26" t="s">
-        <v>55</v>
-      </c>
-      <c r="B14" s="26"/>
-      <c r="C14" s="26"/>
+      <c r="A14" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" s="28"/>
+      <c r="C14" s="28"/>
     </row>
     <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="26" t="s">
-        <v>56</v>
-      </c>
-      <c r="B15" s="26"/>
-      <c r="C15" s="26"/>
+      <c r="A15" s="28" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>